<commit_message>
docs(gtm): atualiza lista de leads da Fase 1 com edicoes mais recentes
Continuacao de 6bdbcf4a — refletia edicoes locais nao commitadas na
planilha antes desta reconciliacao com o origin/main.
</commit_message>
<xml_diff>
--- a/docs/gtm/lista-dos-200-fase1.xlsx
+++ b/docs/gtm/lista-dos-200-fase1.xlsx
@@ -1647,7 +1647,7 @@
       <c r="S3" s="11" t="n"/>
       <c r="T3" s="11" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: sem site.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: sem site. Sem Instagram proprio localizavel via busca - so aparece em agregador (FitFit.Fitness, nota 9,2/10 e 4,4/5). Endereco: Av. Paulo Faccini 691. Abertura generica (sem sinal especifico).</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,11 @@
           <t>Guarulhos - Centro</t>
         </is>
       </c>
-      <c r="D4" s="27" t="n"/>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>@crossfitforvy</t>
+        </is>
+      </c>
       <c r="E4" s="27" t="inlineStr">
         <is>
           <t>+55 11 93394-9736</t>
@@ -1706,7 +1710,7 @@
       <c r="S4" s="27" t="n"/>
       <c r="T4" s="27" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial. Instagram @crossfitforvy, 3 mil seguidores, 511 posts, ativo. Fez Festivus Games em 2026-04.</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1729,11 @@
           <t>Guarulhos - Picanço</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n"/>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>@crossfitmk1</t>
+        </is>
+      </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
           <t>+55 11 98964-7226</t>
@@ -1765,7 +1773,7 @@
       <c r="S5" s="11" t="n"/>
       <c r="T5" s="11" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site próprio.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site proprio. Instagram @crossfitmk1, 11,1 mil seguidores, desde 2012, pioneira em Guarulhos, tem CrossFit Kids. Possivel rede de 2 unidades com a MK1 Vila Galvao (linha 6) - confirmar.</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1792,11 @@
           <t>Guarulhos - Vila Galvão</t>
         </is>
       </c>
-      <c r="D6" s="27" t="n"/>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>@crossfitmk1</t>
+        </is>
+      </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
           <t>+55 11 91223-9182</t>
@@ -1824,7 +1836,7 @@
       <c r="S6" s="27" t="n"/>
       <c r="T6" s="27" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial. Mesma marca/Instagram da MK-1 Picanco (linha 5) - possivel 2a unidade da mesma rede, nao a mesma pessoa necessariamente. Confirmar antes de abordar como lead separado.</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1855,11 @@
           <t>Guarulhos - Vila Rio</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n"/>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>@crossfitsaurus</t>
+        </is>
+      </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
           <t>+55 11 98254-0787</t>
@@ -1883,7 +1899,7 @@
       <c r="S7" s="11" t="n"/>
       <c r="T7" s="11" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site próprio.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site proprio. ATENCAO: parece rede com 3+ unidades (Bosque Maia, Vila Guilherme, Freguesia, possivelmente mais - o mesmo telefone aparece tambem no Tier 2 como "CrossFit Saurus" em Vila Guilherme). Regra do script (secao 6) desqualifica rede com mais de 3 unidades na Fase 1 - confirmar com Renan antes de abordar; se confirmado, marcar Descartado.</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1918,11 @@
           <t>Guarulhos - Vila Augusta</t>
         </is>
       </c>
-      <c r="D8" s="27" t="n"/>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>@crossfitvilaaugusta</t>
+        </is>
+      </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
           <t>+55 11 93022-9182</t>
@@ -1942,7 +1962,7 @@
       <c r="S8" s="27" t="n"/>
       <c r="T8" s="27" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial. Instagram @crossfitvilaaugusta, 1,2 mil seguidores. Comunidade bem ativa: aulao de dia dos pais, churrasco do box, musica ao vivo - perfil familiar/comunitario forte.</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1981,11 @@
           <t>Guarulhos - Vila Augusta</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n"/>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>@cf_gru</t>
+        </is>
+      </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
           <t>+55 11 97246-7271</t>
@@ -2001,7 +2025,7 @@
       <c r="S9" s="11" t="n"/>
       <c r="T9" s="11" t="inlineStr">
         <is>
-          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site próprio.</t>
+          <t>Tier 1 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site proprio. Instagram @cf_gru, 6,1 mil seguidores, 8+ anos de historia. Posta o WOD do dia no feed regularmente (sinal direto da Variante A do script). Tem e-mail proprio (contato@crossfitgru.com).</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2394,11 @@
           <t>São Paulo - Jacana</t>
         </is>
       </c>
-      <c r="D16" s="27" t="n"/>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>@crossfitbatalha</t>
+        </is>
+      </c>
       <c r="E16" s="27" t="inlineStr">
         <is>
           <t>+55 11 94037-4949</t>
@@ -2410,7 +2438,7 @@
       <c r="S16" s="27" t="n"/>
       <c r="T16" s="27" t="inlineStr">
         <is>
-          <t>Tier 2 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial.</t>
+          <t>Tier 2 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial. Instagram @crossfitbatalha, 3,7 mil seguidores, Jacana/zona norte. Posiciona "CrossFit e para TODOS" e agenda aula experimental direto pelo Instagram - fluxo de agendamento manual.</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2516,11 @@
           <t>São Paulo - Mandaqui</t>
         </is>
       </c>
-      <c r="D18" s="27" t="n"/>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>@crossfitbetta</t>
+        </is>
+      </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
           <t>+55 11 2281-9110</t>
@@ -2528,7 +2560,7 @@
       <c r="S18" s="27" t="n"/>
       <c r="T18" s="27" t="inlineStr">
         <is>
-          <t>Tier 2 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial.</t>
+          <t>Tier 2 (varredura TomTom 2026-08-29, PR #185). Qualificacao: afiliado oficial. Instagram @crossfitbetta, quase 4 mil seguidores, Mandaqui. Posicionamento de bem-estar ("saude fisica e mental", "mais que uma academia").</t>
         </is>
       </c>
     </row>
@@ -6956,7 +6988,11 @@
           <t>São Paulo - Tucuruvi</t>
         </is>
       </c>
-      <c r="D94" s="27" t="n"/>
+      <c r="D94" s="27" t="inlineStr">
+        <is>
+          <t>@ct_zn_</t>
+        </is>
+      </c>
       <c r="E94" s="27" t="inlineStr">
         <is>
           <t>+55 11 99906-2601</t>
@@ -6996,7 +7032,7 @@
       <c r="S94" s="27" t="n"/>
       <c r="T94" s="27" t="inlineStr">
         <is>
-          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site próprio.</t>
+          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site proprio. Instagram @ct_zn_, Tucuruvi. Box competitivo - participa de Open e challenges internos. Cuidado: existe outro lead "Crossfit Zn" (linha 113, Santana) com nome parecido mas telefone diferente - nao confundir na abordagem.</t>
         </is>
       </c>
     </row>
@@ -7979,7 +8015,7 @@
       <c r="S111" s="11" t="n"/>
       <c r="T111" s="11" t="inlineStr">
         <is>
-          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: sem site.</t>
+          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: sem site. Instagram pequeno (21 posts), box novo/recente. Faz promocao tipo Black Friday - sinal de sensibilidade a preco e possivel dor de cobranca manual em campanha.</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8133,7 @@
       <c r="S113" s="11" t="n"/>
       <c r="T113" s="11" t="inlineStr">
         <is>
-          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: sem site.</t>
+          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: sem site. Santana, zona norte. Sinal fraco na busca (nome comum, resultados ambiguos com outros "CrossFit ZN") - abertura generica por bairro, nao usar detalhe de outro box por engano.</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8542,7 @@
       <c r="S120" s="27" t="n"/>
       <c r="T120" s="27" t="inlineStr">
         <is>
-          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site próprio.</t>
+          <t>Tier 3 (varredura TomTom 2026-08-29, PR #185). Qualificacao: site proprio. Tucuruvi. Sinal fraco na busca - mas o proprio nome ja diz que atende funcional + crossfit, publico mais amplo que um box crossfit puro.</t>
         </is>
       </c>
     </row>
@@ -12161,15 +12197,15 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B3:H3"/>
     <mergeCell ref="J16:L16"/>
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="B3:H3"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="J9:K9"/>
   </mergeCells>

</xml_diff>